<commit_message>
Reinvio modifica a CDA2 -     - Aggiunto campo ActSite RA ("Right Arm").
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#GENOMEUPSRLXX/GENOMEUP_SRL/JULIAOMIX/2.42/report-checklist.xlsx
+++ b/GATEWAY/A1#111#GENOMEUPSRLXX/GENOMEUP_SRL/JULIAOMIX/2.42/report-checklist.xlsx
@@ -1188,22 +1188,22 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-04-02T18:41:55+02:00</t>
+          <t>2026-04-07T18:27:59+02:00</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>bab0c9784538c959e3c045695fb1f7be</t>
+          <t>6c514731150632507fbc85a2ba3c201d</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.10.1.9.1.5.99f90b33ca75f2590aaa5a93e349a5a4349b644fa2ab89a954ef589df3628360.4f31a33829^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.10.1.9.1.5.99f90b33ca75f2590aaa5a93e349a5a4349b644fa2ab89a954ef589df3628360.4ee24ae845^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1284,22 +1284,22 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-04-02T18:41:55+02:00</t>
+          <t>2026-04-07T18:27:59+02:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>c99c38443ce75a50d2817ae314720404</t>
+          <t>a84dda0b20754c8f594180850e0d7965</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.10.1.9.1.5.7f9944409201df7c089369287091b1000846949ae2d6223a3804b15ba36e4e05.b2d7c9fc1e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.10.1.9.1.5.7f9944409201df7c089369287091b1000846949ae2d6223a3804b15ba36e4e05.2cfad4c7d4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1380,22 +1380,22 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-04-02T18:41:56+02:00</t>
+          <t>2026-04-07T18:28:00+02:00</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>433d02f40facb42d21ff390af07015e2</t>
+          <t>eae5306403f06173dc7e140b414a8c3b</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.10.1.9.1.5.0e5147edbed9fd19dd7ef6d416b05d094581c63dc703d34f8de22423729b4e2b.3b092db2a8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.10.1.9.1.5.0e5147edbed9fd19dd7ef6d416b05d094581c63dc703d34f8de22423729b4e2b.f7d76b90be^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1476,22 +1476,22 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-04-02T18:41:56+02:00</t>
+          <t>2026-04-07T18:28:00+02:00</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>df2ac73d200ebf3f07227c14f733a833</t>
+          <t>8c8e9c030551a7049107a1f35794b207</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.10.1.9.1.5.0ba8c553995218d37f7cbc0fca74ebfc06cb4853aebd725c8036e5332e9e107f.dbcb064a6e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.10.1.9.1.5.0ba8c553995218d37f7cbc0fca74ebfc06cb4853aebd725c8036e5332e9e107f.0a59d14261^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1572,22 +1572,22 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-04-02T18:41:57+02:00</t>
+          <t>2026-04-07T18:28:00+02:00</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>9985248405b526ce639c1dc9b2a70b0c</t>
+          <t>97318948572dd841b16b69a6f10906e5</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.10.1.9.1.5.2b7345a7547f7f21efdffba1cbfd80bbcbe67cbca1aa27123f444151e605c662.6f92b6b421^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.10.1.9.1.5.2b7345a7547f7f21efdffba1cbfd80bbcbe67cbca1aa27123f444151e605c662.0dd79c0d9a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -1668,22 +1668,22 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-04-02T18:41:57+02:00</t>
+          <t>2026-04-07T18:28:01+02:00</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>5cc9fcf7749466d64af1b2da60f5fb03</t>
+          <t>e22fc0fff9f07043d708703df8f32718</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.10.1.9.1.5.d0677696d15a52815c704fce2ee0ec31e21c8786ddbbf475e2b23426e1301525.9fe2d0b43b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.10.1.9.1.5.d0677696d15a52815c704fce2ee0ec31e21c8786ddbbf475e2b23426e1301525.12aeb75129^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1764,22 +1764,22 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-04-02T18:41:58+02:00</t>
+          <t>2026-04-07T18:28:01+02:00</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>5c7ba38b07f77137f70ef098fc33de31</t>
+          <t>fa9e5cfdc8e2722b8513eb07ddc359a0</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.10.1.9.1.5.3532a5903c5cc9504e0b93ab60965b980a2355d02de958d6127651d3b540ef11.6340a7593a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.10.1.9.1.5.3532a5903c5cc9504e0b93ab60965b980a2355d02de958d6127651d3b540ef11.3f73df4ed5^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1860,22 +1860,22 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-04-02T18:41:58+02:00</t>
+          <t>2026-04-07T18:28:02+02:00</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>e20ce0720554121496649af105c088ba</t>
+          <t>6a80395ee5d497c8f21040f6e8ac307b</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.10.1.9.1.5.fdf5d654fa7a532947ad7164396baf0fedc5f8d2e97f7ac10158fac9fd2fcce9.222db56132^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.10.1.9.1.5.fdf5d654fa7a532947ad7164396baf0fedc5f8d2e97f7ac10158fac9fd2fcce9.fee7c4304f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1958,22 +1958,22 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-04-02T18:41:59+02:00</t>
+          <t>2026-04-07T18:32:03+02:00</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>5043ba39a1033a8f5533f6aeee3f55e1</t>
+          <t>6df7355cd281c7a0667171c662f468b5</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.10.1.9.1.5.1c7a566e6fa49ed06131c36e5e27fa198abed46f4665b0548642ccf9ac0a3288.fbb6f5f003^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.10.1.9.1.5.1c7a566e6fa49ed06131c36e5e27fa198abed46f4665b0548642ccf9ac0a3288.3c071d005f^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -2020,22 +2020,22 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-04-02T18:41:59+02:00</t>
+          <t>2026-04-07T18:28:02+02:00</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1fc40379d9db561ececc69b1697c11d5</t>
+          <t>7696e710d3559cceb4ef6fdaa53eb7da</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.10.1.9.1.5.8d319f8888befbf1503b7b35cd5729eb9b5e69fe536f4e8ceaa8e4bbd6a7e4c6.042968ef3e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.10.1.9.1.5.8d319f8888befbf1503b7b35cd5729eb9b5e69fe536f4e8ceaa8e4bbd6a7e4c6.5a647b320d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -2116,22 +2116,22 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-04-02T18:42:00+02:00</t>
+          <t>2026-04-07T18:28:03+02:00</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>781545198526f3b67736017edaf1bab4</t>
+          <t>1c427f4039716746090bcda69407bb53</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.10.1.9.1.5.b1d073a56be0e87ebd69656dc19ee8965f57dc5161aa80ba5a0982cf8345a404.a4ae12a2d2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.10.1.9.1.5.b1d073a56be0e87ebd69656dc19ee8965f57dc5161aa80ba5a0982cf8345a404.7823cd6ade^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">

</xml_diff>